<commit_message>
This is the second commit
</commit_message>
<xml_diff>
--- a/Downloads/Itemised_List_for_Insurance_Updated.xlsx
+++ b/Downloads/Itemised_List_for_Insurance_Updated.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jevap\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7A5E8811-69E5-4B42-9509-B4550E581864}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74A338C6-9E46-47B8-8656-3EA36F581595}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3348" yWindow="3348" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>Total</t>
   </si>
@@ -79,6 +79,9 @@
   </si>
   <si>
     <t>Guitar Amplifier	Fender	Fender Mustang IV v2 Amplifier</t>
+  </si>
+  <si>
+    <t>sample</t>
   </si>
 </sst>
 </file>
@@ -197,10 +200,10 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -492,12 +495,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
     </row>
     <row r="2" spans="1:4" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
@@ -517,7 +520,7 @@
       <c r="A3" s="3">
         <v>1</v>
       </c>
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="11" t="s">
         <v>6</v>
       </c>
       <c r="C3" s="10">
@@ -629,9 +632,15 @@
       <c r="A11" s="3">
         <v>9</v>
       </c>
-      <c r="B11" s="9"/>
-      <c r="C11" s="10"/>
-      <c r="D11" s="8"/>
+      <c r="B11" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C11" s="10">
+        <v>0</v>
+      </c>
+      <c r="D11" s="8">
+        <v>0</v>
+      </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="3">

</xml_diff>